<commit_message>
CAD v7.1-v7.2: soporte estéreo StereoVision_03 y ventosa JXD en el eje hueco
- Cámaras: el soporte StereoVision_03 del usuario (base CB-156 remodelada con
  4 agujeros M3, tapa CB-157) va sobre el adaptador CB-154 en el cabezal del
  mástil; base estéreo de 71 mm. Salen la barra CB-154 y el soporte CB-155.
  Pieza de pruebas CB-158 con bola Ø11,8 para la rótula del trípode y
  conjunto CB-159.
- Herramienta: la punta de CB-606 toma la parte de arriba de la ventosa JXD
  medida (Ø19 con planos a 17) en un alojamiento doble D, así la torsión gira
  la ventosa. El racor 6 mm × G1/4 baja por dentro del eje, apoya en un fondo
  de 3 mm y aprieta la ventosa contra él. Nuevos CB-618 (ventosa), CB-619
  (racor) y CB-620 (llave de montaje); la McMaster CB-617 sale de CB-600.
- STL en cad/imprimir, BOM, docs, vision/config y scripts de la API.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/BOM_CitriBot.xlsx
+++ b/bom/BOM_CitriBot.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$1:$M$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$1:$M$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M107"/>
+  <dimension ref="A1:M112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Visión estéreo, en el mástil CB-150 (a 120 mm entre lentes)</t>
+          <t>Visión estéreo, en el soporte CB-156 del mástil (71 mm entre lentes)</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Precio del pedido 'Cámaras': confirmar si es por unidad o por las dos. CAD: CB-515. Quitarles la pinza de monitor</t>
+          <t>Precio del pedido 'Cámaras': confirmar si es por unidad o por las dos. CAD: CB-515. Se cuelgan con su propia pinza de monitor en la pared del soporte</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>Pedido 'Ventosa 1'</t>
+          <t>Pedido 'Ventosa 1'. Su parte de arriba (Ø19, planos a 17) entra en la punta de CB-606; el racor N03 la aprieta desde adentro. CAD: CB-618 (medida, Ø40 × 22)</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1699,7 @@
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>Pedido 'Ventosa 2'</t>
+          <t>Pedido 'Ventosa 2'. Si su parte de arriba no es igual a la de la N01, no entra en el alojamiento de CB-606</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Macho 1/4 a manguera 6 mm (tipo PC6-02)</t>
+          <t>Recto, manguera 6 mm × rosca macho 1/4" BSP con junta tórica (0,9" de alto)</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
@@ -1758,7 +1758,7 @@
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>Pedido 'Unión neumática'</t>
+          <t>Pedido 'Unión neumática'. CAD: CB-619; medir hexágono (≈ 14), anillo (≈ Ø16,5 × 1,8), cuello (≈ 3) y rosca (≈ 4,5) antes de imprimir CB-606 y CB-620</t>
         </is>
       </c>
     </row>
@@ -3075,7 +3075,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr"/>
       <c r="E49" s="2" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3084,7 +3084,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>3 tapa de E2 → E2 · 4 Sabertooth → bandeja · 8 pestañas de los servos · 2 porta-servo · 4 placa CB-306 → insertos de E2 · 4 soportes C270 → barra estéreo</t>
+          <t>3 tapa de E2 → E2 · 4 Sabertooth → bandeja · 8 pestañas de los servos · 2 porta-servo · 4 placa CB-306 → insertos de E2</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr"/>
       <c r="E50" s="2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3129,7 +3129,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Tapa de la caja de torsión</t>
+          <t>4 tapa de la caja de torsión · 4 base del soporte estéreo CB-156 → adaptador CB-154</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Soportes C270 → barra estéreo</t>
+          <t>Base del soporte estéreo → adaptador CB-154 (en los alojamientos hexagonales)</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -4274,26 +4274,26 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>X01</t>
+          <t>H30</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Materia prima y consumibles</t>
+          <t>Tornillería</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Tablero contrachapado o MDF</t>
+          <t>Tornillo autorroscante Ø3,5 × 10</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>550 × 550 × 16 mm</t>
+          <t>Cabeza plana</t>
         </is>
       </c>
       <c r="E75" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Base del brazo</t>
+          <t>Tapas CB-157 → postes del soporte estéreo (agujeros de Ø3,25)</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -4318,44 +4318,40 @@
       <c r="J75" s="3" t="n"/>
       <c r="K75" s="2" t="inlineStr"/>
       <c r="L75" s="2" t="inlineStr"/>
-      <c r="M75" s="2" t="inlineStr">
-        <is>
-          <t>Agujeros: Ø42 motor J1 y 4 × Ø4.5 bandeja (ver CB-111)</t>
-        </is>
-      </c>
+      <c r="M75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>X02</t>
+          <t>H31</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Materia prima y consumibles</t>
+          <t>Tornillería</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Filamento PETG</t>
+          <t>Tornillo M3 × 25 Allen + tuerca M3</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>1,75 mm</t>
+          <t>DIN 912</t>
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>u</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Piezas impresas</t>
+          <t>Alma del cuello de la bola de la pieza de pruebas CB-158</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -4373,14 +4369,14 @@
       <c r="L76" s="2" t="inlineStr"/>
       <c r="M76" s="2" t="inlineStr">
         <is>
-          <t>Estimado 3–4 kg: calcular con el slicer</t>
+          <t>Solo para las pruebas de visión sin el brazo</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>X03</t>
+          <t>X01</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -4390,10 +4386,14 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Epoxi bicomponente</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr"/>
+          <t>Tablero contrachapado o MDF</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>550 × 550 × 16 mm</t>
+        </is>
+      </c>
       <c r="E77" s="2" t="n">
         <v>1</v>
       </c>
@@ -4404,7 +4404,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Buje D8 en E2 · brida y tapón del tubo de E3</t>
+          <t>Base del brazo</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -4420,12 +4420,16 @@
       <c r="J77" s="3" t="n"/>
       <c r="K77" s="2" t="inlineStr"/>
       <c r="L77" s="2" t="inlineStr"/>
-      <c r="M77" s="2" t="inlineStr"/>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>Agujeros: Ø42 motor J1 y 4 × Ø4.5 bandeja (ver CB-111)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>X04</t>
+          <t>X02</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -4435,21 +4439,25 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Cianoacrilato</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr"/>
+          <t>Filamento PETG</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>1,75 mm</t>
+        </is>
+      </c>
       <c r="E78" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Imán en el soporte CB-232</t>
+          <t>Piezas impresas</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -4465,12 +4473,16 @@
       <c r="J78" s="3" t="n"/>
       <c r="K78" s="2" t="inlineStr"/>
       <c r="L78" s="2" t="inlineStr"/>
-      <c r="M78" s="2" t="inlineStr"/>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>Estimado 3–4 kg: calcular con el slicer</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>X05</t>
+          <t>X03</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -4480,14 +4492,10 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Tubo cuadrado de aluminio</t>
-        </is>
-      </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>30 × 30 × 2 mm, largo 440 mm</t>
-        </is>
-      </c>
+          <t>Epoxi bicomponente</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr"/>
       <c r="E79" s="2" t="n">
         <v>1</v>
       </c>
@@ -4498,7 +4506,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Eslabón E3 (prismático J3)</t>
+          <t>Buje D8 en E2 · brida y tapón del tubo de E3</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -4514,16 +4522,12 @@
       <c r="J79" s="3" t="n"/>
       <c r="K79" s="2" t="inlineStr"/>
       <c r="L79" s="2" t="inlineStr"/>
-      <c r="M79" s="2" t="inlineStr">
-        <is>
-          <t>CAD: CB-401. Se desliza en el canal 31 × 31 de E2: cinta de PTFE (X06)</t>
-        </is>
-      </c>
+      <c r="M79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>X06</t>
+          <t>X04</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -4533,25 +4537,21 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Cinta de PTFE adhesiva</t>
-        </is>
-      </c>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>Ancho ≥ 20 mm</t>
-        </is>
-      </c>
+          <t>Cianoacrilato</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr"/>
       <c r="E80" s="2" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>u</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Canal 31 × 31 de E2 (guía de J3)</t>
+          <t>Imán en el soporte CB-232</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -4572,7 +4572,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>X07</t>
+          <t>X05</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -4582,16 +4582,16 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Precinto plástico</t>
+          <t>Tubo cuadrado de aluminio</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>≈ 3 mm de ancho</t>
+          <t>30 × 30 × 2 mm, largo 440 mm</t>
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4600,7 +4600,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>2 extremos de la correa de J3 en la pinza CB-403 · 2 cámaras C270 en sus soportes</t>
+          <t>Eslabón E3 (prismático J3)</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -4616,12 +4616,16 @@
       <c r="J81" s="3" t="n"/>
       <c r="K81" s="2" t="inlineStr"/>
       <c r="L81" s="2" t="inlineStr"/>
-      <c r="M81" s="2" t="inlineStr"/>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>CAD: CB-401. Se desliza en el canal 31 × 31 de E2: cinta de PTFE (X06)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>X08</t>
+          <t>X06</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -4631,25 +4635,25 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Tubo cuadrado de aluminio</t>
+          <t>Cinta de PTFE adhesiva</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>20 × 20 × 1,5 mm, largo 627 mm</t>
+          <t>Ancho ≥ 20 mm</t>
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Mástil de las cámaras</t>
+          <t>Canal 31 × 31 de E2 (guía de J3)</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
@@ -4665,45 +4669,45 @@
       <c r="J82" s="3" t="n"/>
       <c r="K82" s="2" t="inlineStr"/>
       <c r="L82" s="2" t="inlineStr"/>
-      <c r="M82" s="2" t="inlineStr">
-        <is>
-          <t>CAD: CB-152</t>
-        </is>
-      </c>
+      <c r="M82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>P01</t>
+          <t>X07</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Piezas impresas</t>
+          <t>Materia prima y consumibles</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>CB-112 Pata de la base</t>
+          <t>Precinto plástico</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>PETG, ≥ 4 perímetros</t>
+          <t>≈ 3 mm de ancho</t>
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
           <t>u</t>
         </is>
       </c>
-      <c r="G83" s="2" t="inlineStr"/>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Extremos de la correa de J3 en la pinza CB-403</t>
+        </is>
+      </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Impresión 3D</t>
+          <t>Por comprar</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
@@ -4712,33 +4716,29 @@
         </is>
       </c>
       <c r="J83" s="3" t="n"/>
-      <c r="K83" s="2" t="inlineStr">
-        <is>
-          <t>Impresora del grupo (Ender 3 V2)</t>
-        </is>
-      </c>
+      <c r="K83" s="2" t="inlineStr"/>
       <c r="L83" s="2" t="inlineStr"/>
       <c r="M83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>X08</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Piezas impresas</t>
+          <t>Materia prima y consumibles</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>CB-121 Placa fija J1 (1M2A)</t>
+          <t>Tubo cuadrado de aluminio</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>PETG, ≥ 4 perímetros</t>
+          <t>20 × 20 × 1,5 mm, largo 627 mm</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
@@ -4749,10 +4749,14 @@
           <t>u</t>
         </is>
       </c>
-      <c r="G84" s="2" t="inlineStr"/>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Mástil de las cámaras</t>
+        </is>
+      </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>Impresión 3D</t>
+          <t>Por comprar</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
@@ -4761,18 +4765,18 @@
         </is>
       </c>
       <c r="J84" s="3" t="n"/>
-      <c r="K84" s="2" t="inlineStr">
-        <is>
-          <t>Impresora del grupo (Ender 3 V2)</t>
-        </is>
-      </c>
+      <c r="K84" s="2" t="inlineStr"/>
       <c r="L84" s="2" t="inlineStr"/>
-      <c r="M84" s="2" t="inlineStr"/>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>CAD: CB-152</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>P01</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -4782,7 +4786,7 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>CB-131 Soporte motor J1 (37D)</t>
+          <t>CB-112 Pata de la base</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -4791,7 +4795,7 @@
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4821,7 +4825,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4831,7 +4835,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>CB-141 Bandeja de electrónica</t>
+          <t>CB-121 Placa fija J1 (1M2A)</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -4865,16 +4869,12 @@
         </is>
       </c>
       <c r="L86" s="2" t="inlineStr"/>
-      <c r="M86" s="2" t="inlineStr">
-        <is>
-          <t>210 × 100 mm</t>
-        </is>
-      </c>
+      <c r="M86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P03</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>CB-201 Plato giratorio con dientes T5 (1M1B)</t>
+          <t>CB-131 Soporte motor J1 (37D)</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -4923,7 +4923,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>P06</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>CB-210 Torre de cintura (2M1D mod)</t>
+          <t>CB-141 Bandeja de electrónica</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -4969,14 +4969,14 @@
       <c r="L88" s="2" t="inlineStr"/>
       <c r="M88" s="2" t="inlineStr">
         <is>
-          <t>318 mm de alto: hay que partirla para la Ender 3 V2</t>
+          <t>210 × 100 mm</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -4986,7 +4986,7 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>CB-232 Soporte del imán</t>
+          <t>CB-201 Plato giratorio con dientes T5 (1M1B)</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -5025,7 +5025,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P06</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -5035,12 +5035,12 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>CB-301 Eslabón E2</t>
+          <t>CB-210 Torre de cintura (2M1D mod)</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>PETG: cubo ≥ 6 perímetros 50 %, cola 3 perímetros 15 %</t>
+          <t>PETG, ≥ 4 perímetros</t>
         </is>
       </c>
       <c r="E90" s="2" t="n">
@@ -5071,14 +5071,14 @@
       <c r="L90" s="2" t="inlineStr"/>
       <c r="M90" s="2" t="inlineStr">
         <is>
-          <t>470 mm de largo: partir en 2 tramos (cubo del hombro hasta x ≈ −100 + cola). La cola liviana baja el torque de J2</t>
+          <t>318 mm de alto: hay que partirla para la Ender 3 V2</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>CB-402 Brida de E3 (herramienta)</t>
+          <t>CB-232 Soporte del imán</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -5122,16 +5122,12 @@
         </is>
       </c>
       <c r="L91" s="2" t="inlineStr"/>
-      <c r="M91" s="2" t="inlineStr">
-        <is>
-          <t>Tapón al 100 % de relleno</t>
-        </is>
-      </c>
+      <c r="M91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -5141,12 +5137,12 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>CB-303 Tapa de E2 / soporte AS5600</t>
+          <t>CB-301 Eslabón E2</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>PETG, ≥ 4 perímetros</t>
+          <t>PETG: cubo ≥ 6 perímetros 50 %, cola 3 perímetros 15 %</t>
         </is>
       </c>
       <c r="E92" s="2" t="n">
@@ -5175,12 +5171,16 @@
         </is>
       </c>
       <c r="L92" s="2" t="inlineStr"/>
-      <c r="M92" s="2" t="inlineStr"/>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>470 mm de largo: partir en 2 tramos (cubo del hombro hasta x ≈ −100 + cola). La cola liviana baja el torque de J2</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>CB-305 Buje D8 del hombro</t>
+          <t>CB-402 Brida de E3 (herramienta)</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -5226,14 +5226,14 @@
       <c r="L93" s="2" t="inlineStr"/>
       <c r="M93" s="2" t="inlineStr">
         <is>
-          <t>Mejor en aluminio: transmite el torque del hombro (≈ 39 kg·cm de pico)</t>
+          <t>Tapón al 100 % de relleno</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>CB-403 Tapón trasero con pinza de correa</t>
+          <t>CB-303 Tapa de E2 / soporte AS5600</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -5277,16 +5277,12 @@
         </is>
       </c>
       <c r="L94" s="2" t="inlineStr"/>
-      <c r="M94" s="2" t="inlineStr">
-        <is>
-          <t>Relleno 100 %</t>
-        </is>
-      </c>
+      <c r="M94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -5296,7 +5292,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>CB-601 Horquilla U</t>
+          <t>CB-305 Buje D8 del hombro</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -5330,12 +5326,16 @@
         </is>
       </c>
       <c r="L95" s="2" t="inlineStr"/>
-      <c r="M95" s="2" t="inlineStr"/>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>Mejor en aluminio: transmite el torque del hombro (≈ 39 kg·cm de pico)</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -5345,7 +5345,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>CB-602 Porta-servo</t>
+          <t>CB-403 Tapón trasero con pinza de correa</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -5379,12 +5379,16 @@
         </is>
       </c>
       <c r="L96" s="2" t="inlineStr"/>
-      <c r="M96" s="2" t="inlineStr"/>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>Relleno 100 %</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -5394,7 +5398,7 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>CB-603 Caja de torsión</t>
+          <t>CB-601 Horquilla U</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -5433,7 +5437,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -5443,7 +5447,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>CB-604 Tapa de la caja</t>
+          <t>CB-602 Porta-servo</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -5482,7 +5486,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -5492,7 +5496,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>CB-605 Polea del servo GT2 66 dientes</t>
+          <t>CB-603 Caja de torsión</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -5526,16 +5530,12 @@
         </is>
       </c>
       <c r="L99" s="2" t="inlineStr"/>
-      <c r="M99" s="2" t="inlineStr">
-        <is>
-          <t>Relleno 100 %</t>
-        </is>
-      </c>
+      <c r="M99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>P18</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -5545,7 +5545,7 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>CB-606 Eje hueco con polea GT2 66 dientes</t>
+          <t>CB-604 Tapa de la caja</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -5579,16 +5579,12 @@
         </is>
       </c>
       <c r="L100" s="2" t="inlineStr"/>
-      <c r="M100" s="2" t="inlineStr">
-        <is>
-          <t>Relleno 100 %</t>
-        </is>
-      </c>
+      <c r="M100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -5598,7 +5594,7 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>CB-607 Separador del pivote</t>
+          <t>CB-605 Polea del servo GT2 66 dientes</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -5632,12 +5628,16 @@
         </is>
       </c>
       <c r="L101" s="2" t="inlineStr"/>
-      <c r="M101" s="2" t="inlineStr"/>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>Relleno 100 %</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -5647,7 +5647,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Anillo de retención del eje hueco</t>
+          <t>CB-606 Eje hueco con polea GT2 66 dientes</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -5683,14 +5683,14 @@
       <c r="L102" s="2" t="inlineStr"/>
       <c r="M102" s="2" t="inlineStr">
         <is>
-          <t>Solo en el .scad (pieza 5), no en el STEP de la herramienta</t>
+          <t>Relleno 100 %. Alojamiento doble D para la ventosa en la punta (el eje gira la ventosa) y fondo de 3 mm donde apoya el racor N03. Imprimir con la polea abajo, sin soportes. STL: cad/imprimir/CB-606_Eje_Hueco_Polea.stl</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -5700,7 +5700,7 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>CB-306 Placa soporte del NEMA 17 (J3)</t>
+          <t>CB-607 Separador del pivote</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -5734,16 +5734,12 @@
         </is>
       </c>
       <c r="L103" s="2" t="inlineStr"/>
-      <c r="M103" s="2" t="inlineStr">
-        <is>
-          <t>Relleno 100 %. Va a E2 con 4 insertos M3 (H26)</t>
-        </is>
-      </c>
+      <c r="M103" s="2" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -5753,7 +5749,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>CB-151 Pie del mástil de las cámaras</t>
+          <t>Anillo de retención del eje hueco</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -5789,14 +5785,14 @@
       <c r="L104" s="2" t="inlineStr"/>
       <c r="M104" s="2" t="inlineStr">
         <is>
-          <t>Relleno 100 %</t>
+          <t>Solo en el .scad (pieza 5), no en el STEP de la herramienta</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -5806,7 +5802,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>CB-153 Cabezal del mástil</t>
+          <t>CB-306 Placa soporte del NEMA 17 (J3)</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -5842,14 +5838,14 @@
       <c r="L105" s="2" t="inlineStr"/>
       <c r="M105" s="2" t="inlineStr">
         <is>
-          <t>Relleno 100 %. Orejas del pivote de cabeceo M5</t>
+          <t>Relleno 100 %. Va a E2 con 4 insertos M3 (H26)</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -5859,7 +5855,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>CB-154 Barra estéreo</t>
+          <t>CB-151 Pie del mástil de las cámaras</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -5895,14 +5891,14 @@
       <c r="L106" s="2" t="inlineStr"/>
       <c r="M106" s="2" t="inlineStr">
         <is>
-          <t>Relleno 100 %: tiene que ser rígida (si se tuerce hay que recalibrar)</t>
+          <t>Relleno 100 %</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -5912,7 +5908,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>CB-155 Soporte de la C270</t>
+          <t>CB-153 Cabezal del mástil</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -5921,7 +5917,7 @@
         </is>
       </c>
       <c r="E107" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -5946,10 +5942,287 @@
         </is>
       </c>
       <c r="L107" s="2" t="inlineStr"/>
-      <c r="M107" s="2" t="inlineStr"/>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>Relleno 100 %. Orejas del pivote de cabeceo M5</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>P24</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Piezas impresas</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>CB-154 Adaptador del soporte estéreo</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>PETG, ≥ 4 perímetros</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr"/>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>Impresión 3D</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="J108" s="3" t="n"/>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t>Impresora del grupo (Ender 3 V2)</t>
+        </is>
+      </c>
+      <c r="L108" s="2" t="inlineStr"/>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>Relleno 100 %. Une el pivote del cabezal con la base del soporte. STL: cad/imprimir/CB-154_Adaptador_Soporte_Estereo.stl</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>P25</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Piezas impresas</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>CB-156 Base del soporte estéreo (StereoVision_03)</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>PETG, ≥ 4 perímetros</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr"/>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Impresión 3D</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="J109" s="3" t="n"/>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t>Impresora del grupo (Ender 3 V2)</t>
+        </is>
+      </c>
+      <c r="L109" s="2" t="inlineStr"/>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>Remodelada del STL del usuario con los 4 agujeros para el adaptador ya hechos. STL: cad/imprimir/CB-156_Soporte_Estereo_C270_Base.stl</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>P26</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Piezas impresas</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>CB-157 Tapa del soporte estéreo</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>PETG, ≥ 4 perímetros</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr"/>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>Impresión 3D</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="J110" s="3" t="n"/>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t>Impresora del grupo (Ender 3 V2)</t>
+        </is>
+      </c>
+      <c r="L110" s="2" t="inlineStr"/>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>Traba la pinza de cada C270. STL: cad/imprimir/CB-157_Soporte_Estereo_C270_Tapa.stl</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>P27</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Piezas impresas</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>CB-158 Adaptador con bola para la rótula del trípode (pruebas)</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>PETG, 4 perímetros, 50 %</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>Probar las cámaras en el trípode antes de montar el brazo</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>Impresión 3D</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="J111" s="3" t="n"/>
+      <c r="K111" s="2" t="inlineStr">
+        <is>
+          <t>Impresora del grupo (Ender 3 V2)</t>
+        </is>
+      </c>
+      <c r="L111" s="2" t="inlineStr"/>
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>No va en el robot. Bola Ø11,8 y cuello Ø4,8 en lugar del perno M6 del trípode; se cambia por CB-154 sin tocar las cámaras. Imprimir con la cara de arriba en la cama y soportes bajo la bola. STL: cad/imprimir/CB-158_Adaptador_Rotula_Bola12.stl</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>P28</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Piezas impresas</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>CB-620 Llave de montaje del racor (herramienta)</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>PETG, 4 perímetros, 50 %</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>Apretar el racor N03 contra la ventosa desde el lado de la polea</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>Impresión 3D</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="J112" s="3" t="n"/>
+      <c r="K112" s="2" t="inlineStr">
+        <is>
+          <t>Impresora del grupo (Ender 3 V2)</t>
+        </is>
+      </c>
+      <c r="L112" s="2" t="inlineStr"/>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>No va en el robot. STL: cad/imprimir/CB-620_Llave_Montaje_Racor.stl</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M107"/>
+  <autoFilter ref="A1:M112"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Imprimir: un STL por pieza, en carpetas como el CAD
- cad/imprimir separado por subconjunto como cad/solidworks; la herramienta
  va primero (00_Herramienta = 09_Herramienta del CAD).
- STL nuevos de todas las piezas impresas de la BOM que faltaban (base,
  cintura, hombro, prismático y herramienta); se mueven los que ya estaban.
- README de imprimir con cantidades y notas por pieza. CB-210 (318 mm de
  alto) y CB-301 (470 mm de largo) no entran en la Ender 3 V2.
- Rutas de los STL corregidas en la BOM, el README del CAD y el de visión.
- Script ExportStl.cs para volver a exportarlos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/BOM_CitriBot.xlsx
+++ b/bom/BOM_CitriBot.xlsx
@@ -5683,7 +5683,7 @@
       <c r="L102" s="2" t="inlineStr"/>
       <c r="M102" s="2" t="inlineStr">
         <is>
-          <t>Relleno 100 %. Alojamiento doble D para la ventosa en la punta (el eje gira la ventosa) y fondo de 3 mm donde apoya el racor N03. Imprimir con la polea abajo, sin soportes. STL: cad/imprimir/CB-606_Eje_Hueco_Polea.stl</t>
+          <t>Relleno 100 %. Alojamiento doble D para la ventosa en la punta (el eje gira la ventosa) y fondo de 3 mm donde apoya el racor N03. Imprimir con la polea abajo, sin soportes. STL: cad/imprimir/00_Herramienta/CB-606_Eje_Hueco_Polea.stl</t>
         </is>
       </c>
     </row>
@@ -5997,7 +5997,7 @@
       <c r="L108" s="2" t="inlineStr"/>
       <c r="M108" s="2" t="inlineStr">
         <is>
-          <t>Relleno 100 %. Une el pivote del cabezal con la base del soporte. STL: cad/imprimir/CB-154_Adaptador_Soporte_Estereo.stl</t>
+          <t>Relleno 100 %. Une el pivote del cabezal con la base del soporte. STL: cad/imprimir/01_Base_J0/CB-154_Adaptador_Soporte_Estereo.stl</t>
         </is>
       </c>
     </row>
@@ -6050,7 +6050,7 @@
       <c r="L109" s="2" t="inlineStr"/>
       <c r="M109" s="2" t="inlineStr">
         <is>
-          <t>Remodelada del STL del usuario con los 4 agujeros para el adaptador ya hechos. STL: cad/imprimir/CB-156_Soporte_Estereo_C270_Base.stl</t>
+          <t>Remodelada del STL del usuario con los 4 agujeros para el adaptador ya hechos. STL: cad/imprimir/01_Base_J0/CB-156_Soporte_Estereo_C270_Base.stl</t>
         </is>
       </c>
     </row>
@@ -6103,7 +6103,7 @@
       <c r="L110" s="2" t="inlineStr"/>
       <c r="M110" s="2" t="inlineStr">
         <is>
-          <t>Traba la pinza de cada C270. STL: cad/imprimir/CB-157_Soporte_Estereo_C270_Tapa.stl</t>
+          <t>Traba la pinza de cada C270. STL: cad/imprimir/01_Base_J0/CB-157_Soporte_Estereo_C270_Tapa.stl</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6160,7 @@
       <c r="L111" s="2" t="inlineStr"/>
       <c r="M111" s="2" t="inlineStr">
         <is>
-          <t>No va en el robot. Bola Ø11,8 y cuello Ø4,8 en lugar del perno M6 del trípode; se cambia por CB-154 sin tocar las cámaras. Imprimir con la cara de arriba en la cama y soportes bajo la bola. STL: cad/imprimir/CB-158_Adaptador_Rotula_Bola12.stl</t>
+          <t>No va en el robot. Bola Ø11,8 y cuello Ø4,8 en lugar del perno M6 del trípode; se cambia por CB-154 sin tocar las cámaras. Imprimir con la cara de arriba en la cama y soportes bajo la bola. STL: cad/imprimir/12_Pruebas/CB-158_Adaptador_Rotula_Bola12.stl</t>
         </is>
       </c>
     </row>
@@ -6217,7 +6217,7 @@
       <c r="L112" s="2" t="inlineStr"/>
       <c r="M112" s="2" t="inlineStr">
         <is>
-          <t>No va en el robot. STL: cad/imprimir/CB-620_Llave_Montaje_Racor.stl</t>
+          <t>No va en el robot. STL: cad/imprimir/00_Herramienta/CB-620_Llave_Montaje_Racor.stl</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Herramienta: ranura para el cable del servo de torsión y guía de montaje
- CB-602 porta-servo: ranura de 6,6 mm en la pared del lado del cable para
  que entre el MG996R de torsión con su pasacables; los agujeros de las
  orejas de ese lado se corren 0,6 mm hacia afuera. El cable sale por la
  muesca que ya tenía la caja CB-603. STL nuevo en cad/imprimir.
- docs/montaje_herramienta.md: orden de armado de CB-600, tornillería y
  lámina con la vista explotada rotulada y la herramienta armada.
- README del CAD (§6.13), BOM e imprimir actualizados; script CableServo.cs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bom/BOM_CitriBot.xlsx
+++ b/bom/BOM_CitriBot.xlsx
@@ -5481,7 +5481,11 @@
         </is>
       </c>
       <c r="L98" s="2" t="inlineStr"/>
-      <c r="M98" s="2" t="inlineStr"/>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>Ranura para el cable del servo de torsión (v7.3); el cable sale por la muesca de la caja CB-603. STL: cad/imprimir/00_Herramienta/CB-602_Porta_Servo.stl</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">

</xml_diff>